<commit_message>
Compacta la tarjeta de Disponibilidad global y afina el análisis por rango
- Modal de Disponibilidad global: tarjeta resumen y gráfica reducidas para
  que el análisis se vea sin scroll a 1280x800 (245px -> 55px de scroll).
- narrarSeries menciona ahora el valor más bajo del rango aunque cumpla la
  meta (antes solo se reportaban incumplimientos), para no callar
  variaciones como el 99,9% de un indicador en un mes puntual.
- Reordena Logros_Clientes_Junio_2026_1 (1).xlsx a Insumos/ y suma la
  transcripción de la sesión (transcript.docx).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Insumos/Disponibilidad Consolidado Mayo.xlsx
+++ b/Insumos/Disponibilidad Consolidado Mayo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yordypardopajaro/Proyectos/InformeAccionFiduciariaRemake/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yordypardopajaro/Proyectos/InformeAccionFiduciariaRemake/Insumos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7293CD16-4EE5-0047-B271-83AA5154E268}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D19B93B-C97C-6341-B3C5-8FEA735B4901}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="780" windowWidth="36000" windowHeight="22600" activeTab="5" xr2:uid="{503FB679-EDCF-495D-8857-2B7034316040}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="22600" activeTab="3" xr2:uid="{503FB679-EDCF-495D-8857-2B7034316040}"/>
   </bookViews>
   <sheets>
     <sheet name="Disponibilidad" sheetId="1" r:id="rId1"/>
@@ -8138,8 +8138,8 @@
     <col min="13" max="13" width="7" hidden="1" customWidth="1"/>
     <col min="14" max="14" width="6.5" hidden="1" customWidth="1"/>
     <col min="15" max="15" width="7" hidden="1" customWidth="1"/>
-    <col min="16" max="16" width="6.6640625" hidden="1" customWidth="1"/>
-    <col min="17" max="17" width="7.1640625" hidden="1" customWidth="1"/>
+    <col min="16" max="16" width="6" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="7" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="6.1640625" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="6.6640625" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="6.1640625" bestFit="1" customWidth="1"/>
@@ -9873,11 +9873,11 @@
   <cols>
     <col min="1" max="1" width="11.5" style="24"/>
     <col min="2" max="2" width="42.6640625" style="24" customWidth="1"/>
-    <col min="3" max="3" width="7.6640625" style="24" bestFit="1" customWidth="1"/>
-    <col min="4" max="8" width="0" style="24" hidden="1" customWidth="1"/>
-    <col min="9" max="9" width="7.33203125" style="24" hidden="1" customWidth="1"/>
-    <col min="10" max="10" width="7.6640625" style="24" hidden="1" customWidth="1"/>
-    <col min="11" max="11" width="7.1640625" style="24" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7" style="24" bestFit="1" customWidth="1"/>
+    <col min="4" max="7" width="0" style="24" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="0.1640625" style="24" hidden="1" customWidth="1"/>
+    <col min="9" max="9" width="6.5" style="24" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="7.1640625" style="24" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="8" style="24" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="7.1640625" style="24" bestFit="1" customWidth="1"/>
     <col min="14" max="16384" width="11.5" style="24"/>
@@ -12496,6 +12496,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101001135E4B32B26B2488E4442E57864EA4F" ma:contentTypeVersion="6" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="b283d4cf1c86539e4ae346c38fc01d16">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="dfc41998-78bc-4c08-91de-816c175871b0" xmlns:ns3="a9965282-d0c8-47ef-8054-6f808d6dcc09" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="bac0b173bf2479e8baedba564e5da120" ns2:_="" ns3:_="">
     <xsd:import namespace="dfc41998-78bc-4c08-91de-816c175871b0"/>
@@ -12672,22 +12687,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{49C11C1E-6202-4831-8769-B2E74E43D623}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8EAC4F93-78ED-4936-9AB0-B4C18B11836D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="dfc41998-78bc-4c08-91de-816c175871b0"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="a9965282-d0c8-47ef-8054-6f808d6dcc09"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38B409F7-5C82-4AE4-90D8-6B399D43C457}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -12704,29 +12729,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{49C11C1E-6202-4831-8769-B2E74E43D623}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8EAC4F93-78ED-4936-9AB0-B4C18B11836D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="dfc41998-78bc-4c08-91de-816c175871b0"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="a9965282-d0c8-47ef-8054-6f808d6dcc09"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>